<commit_message>
configure frontend api environment
</commit_message>
<xml_diff>
--- a/backend/output/IndustrialIQ_Enriched_Catalog.xlsx
+++ b/backend/output/IndustrialIQ_Enriched_Catalog.xlsx
@@ -534,7 +534,11 @@
           <t>Rheem Manufacturing</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>sdfasd</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Built-In Dishwashers</t>
@@ -567,14 +571,14 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="M2" t="b">
         <v>1</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -646,7 +650,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -684,12 +688,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>dewlat</t>
+          <t>DEWALT®</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>milwaukee</t>
+          <t>Line Lasers</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -719,7 +723,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="M4" t="b">
         <v>1</v>
@@ -788,11 +792,11 @@
         <v>70</v>
       </c>
       <c r="M5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="O5" t="inlineStr"/>

</xml_diff>